<commit_message>
Integra insumos ubigeo_UGEL y PEIP_solomant
- Usa ubigeo_UGEL.xlsx como insumo geografico: agrega columnas DRE y UGEL a
  todas las bases (cobertura 99.0%).
- df_peip_mantenimiento ahora lee PEIP_solomant.xlsx (separa cui y cod_local);
  pasa de 0% a 100% de cruce con ubigeo.
- Regenera bases limpias por grupo, base final armonizada/union y diccionario.

https://claude.ai/code/session_01N9afypBcQVKYhttom8P34Z
</commit_message>
<xml_diff>
--- a/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_anexo2_b.xlsx
+++ b/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_anexo2_b.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC207"/>
+  <dimension ref="A1:AE207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,6 +566,16 @@
           <t>ubigeo</t>
         </is>
       </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>dre</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>ugel</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -679,6 +689,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -792,6 +812,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -903,6 +933,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1016,6 +1056,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1129,6 +1179,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1244,6 +1304,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1357,6 +1427,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1470,6 +1550,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1583,6 +1673,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1696,6 +1796,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1809,6 +1919,16 @@
           <t>010202</t>
         </is>
       </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1918,6 +2038,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2029,6 +2159,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2142,6 +2282,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2261,6 +2411,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2372,6 +2532,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2485,6 +2655,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2600,6 +2780,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2711,6 +2901,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2824,6 +3024,16 @@
           <t>010201</t>
         </is>
       </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2937,6 +3147,16 @@
           <t>010203</t>
         </is>
       </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3050,6 +3270,16 @@
           <t>010203</t>
         </is>
       </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3163,6 +3393,16 @@
           <t>010204</t>
         </is>
       </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3276,6 +3516,16 @@
           <t>010204</t>
         </is>
       </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3389,6 +3639,16 @@
           <t>010206</t>
         </is>
       </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3502,6 +3762,16 @@
           <t>010206</t>
         </is>
       </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3615,6 +3885,16 @@
           <t>010206</t>
         </is>
       </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3728,6 +4008,16 @@
           <t>010206</t>
         </is>
       </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3843,6 +4133,16 @@
           <t>010206</t>
         </is>
       </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -3954,6 +4254,16 @@
           <t>010206</t>
         </is>
       </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4067,6 +4377,16 @@
           <t>010206</t>
         </is>
       </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -4180,6 +4500,16 @@
           <t>010206</t>
         </is>
       </c>
+      <c r="AD33" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4291,6 +4621,16 @@
       <c r="AC34" t="inlineStr">
         <is>
           <t>010206</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>UGEL BAGUA</t>
         </is>
       </c>
     </row>
@@ -4388,6 +4728,16 @@
       <c r="AC35" t="inlineStr">
         <is>
           <t>010111</t>
+        </is>
+      </c>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>DRE AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr">
+        <is>
+          <t>UGEL CHACHAPOYAS</t>
         </is>
       </c>
     </row>
@@ -4477,6 +4827,16 @@
           <t>021001</t>
         </is>
       </c>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>DRE ANCASH</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>UGEL HUARI</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -4580,6 +4940,16 @@
           <t>021604</t>
         </is>
       </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>DRE ANCASH</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>UGEL POMABAMBA</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -4687,6 +5057,16 @@
           <t>030603</t>
         </is>
       </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>DRE APURIMAC</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>UGEL CHINCHEROS</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -4794,6 +5174,16 @@
           <t>030603</t>
         </is>
       </c>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>DRE APURIMAC</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr">
+        <is>
+          <t>UGEL CHINCHEROS</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -4903,6 +5293,16 @@
           <t>030603</t>
         </is>
       </c>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>DRE APURIMAC</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr">
+        <is>
+          <t>UGEL CHINCHEROS</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -5010,6 +5410,16 @@
           <t>030603</t>
         </is>
       </c>
+      <c r="AD41" t="inlineStr">
+        <is>
+          <t>DRE APURIMAC</t>
+        </is>
+      </c>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>UGEL CHINCHEROS</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -5119,6 +5529,16 @@
           <t>030603</t>
         </is>
       </c>
+      <c r="AD42" t="inlineStr">
+        <is>
+          <t>DRE APURIMAC</t>
+        </is>
+      </c>
+      <c r="AE42" t="inlineStr">
+        <is>
+          <t>UGEL CHINCHEROS</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -5224,6 +5644,16 @@
       <c r="AC43" t="inlineStr">
         <is>
           <t>030603</t>
+        </is>
+      </c>
+      <c r="AD43" t="inlineStr">
+        <is>
+          <t>DRE APURIMAC</t>
+        </is>
+      </c>
+      <c r="AE43" t="inlineStr">
+        <is>
+          <t>UGEL CHINCHEROS</t>
         </is>
       </c>
     </row>
@@ -5321,6 +5751,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD44" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE44" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -5416,6 +5856,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD45" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE45" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -5511,6 +5961,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD46" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE46" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -5606,6 +6066,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD47" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE47" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -5701,6 +6171,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD48" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE48" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -5796,6 +6276,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD49" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE49" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -5891,6 +6381,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD50" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE50" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -5986,6 +6486,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD51" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE51" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -6081,6 +6591,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE52" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -6176,6 +6696,16 @@
           <t>040302</t>
         </is>
       </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>GRE AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AE53" t="inlineStr">
+        <is>
+          <t>UGEL CARAVELI</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -6291,6 +6821,16 @@
       <c r="AC54" t="inlineStr">
         <is>
           <t>050201</t>
+        </is>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE54" t="inlineStr">
+        <is>
+          <t>UGEL CANGALLO</t>
         </is>
       </c>
     </row>
@@ -6384,6 +6924,16 @@
           <t>050604</t>
         </is>
       </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE55" t="inlineStr">
+        <is>
+          <t>UGEL LUCANAS</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -6473,6 +7023,16 @@
       <c r="AC56" t="inlineStr">
         <is>
           <t>050604</t>
+        </is>
+      </c>
+      <c r="AD56" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE56" t="inlineStr">
+        <is>
+          <t>UGEL LUCANAS</t>
         </is>
       </c>
     </row>
@@ -6558,6 +7118,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD57" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE57" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -6641,6 +7211,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD58" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE58" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -6724,6 +7304,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD59" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE59" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -6807,6 +7397,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD60" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE60" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -6890,6 +7490,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD61" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE61" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -6973,6 +7583,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD62" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE62" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -7056,6 +7676,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE63" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -7139,6 +7769,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE64" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -7222,6 +7862,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -7305,6 +7955,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD66" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE66" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -7388,6 +8048,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD67" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE67" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -7471,6 +8141,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD68" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE68" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -7554,6 +8234,16 @@
           <t>050504</t>
         </is>
       </c>
+      <c r="AD69" t="inlineStr">
+        <is>
+          <t>DRE AYACUCHO</t>
+        </is>
+      </c>
+      <c r="AE69" t="inlineStr">
+        <is>
+          <t>UGEL LA MAR</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -7647,6 +8337,16 @@
           <t>070107</t>
         </is>
       </c>
+      <c r="AD70" t="inlineStr">
+        <is>
+          <t>DRE CALLAO</t>
+        </is>
+      </c>
+      <c r="AE70" t="inlineStr">
+        <is>
+          <t>UGEL VENTANILLA</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -7754,6 +8454,16 @@
           <t>070107</t>
         </is>
       </c>
+      <c r="AD71" t="inlineStr">
+        <is>
+          <t>DRE CALLAO</t>
+        </is>
+      </c>
+      <c r="AE71" t="inlineStr">
+        <is>
+          <t>UGEL VENTANILLA</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -7853,6 +8563,16 @@
       <c r="AC72" t="inlineStr">
         <is>
           <t>070107</t>
+        </is>
+      </c>
+      <c r="AD72" t="inlineStr">
+        <is>
+          <t>DRE CALLAO</t>
+        </is>
+      </c>
+      <c r="AE72" t="inlineStr">
+        <is>
+          <t>UGEL VENTANILLA</t>
         </is>
       </c>
     </row>
@@ -7952,6 +8672,16 @@
           <t>070107</t>
         </is>
       </c>
+      <c r="AD73" t="inlineStr">
+        <is>
+          <t>DRE CALLAO</t>
+        </is>
+      </c>
+      <c r="AE73" t="inlineStr">
+        <is>
+          <t>UGEL VENTANILLA</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -8055,6 +8785,16 @@
           <t>100109</t>
         </is>
       </c>
+      <c r="AD74" t="inlineStr">
+        <is>
+          <t>DRE HUANUCO</t>
+        </is>
+      </c>
+      <c r="AE74" t="inlineStr">
+        <is>
+          <t>UGEL HUÁNUCO</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -8152,6 +8892,16 @@
           <t>130905</t>
         </is>
       </c>
+      <c r="AD75" t="inlineStr">
+        <is>
+          <t>GRE LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="AE75" t="inlineStr">
+        <is>
+          <t>UGEL SÁNCHEZ CARRIÓN</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -8273,6 +9023,16 @@
       <c r="AC76" t="inlineStr">
         <is>
           <t>130905</t>
+        </is>
+      </c>
+      <c r="AD76" t="inlineStr">
+        <is>
+          <t>GRE LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="AE76" t="inlineStr">
+        <is>
+          <t>UGEL SÁNCHEZ CARRIÓN</t>
         </is>
       </c>
     </row>
@@ -8368,6 +9128,16 @@
           <t>130905</t>
         </is>
       </c>
+      <c r="AD77" t="inlineStr">
+        <is>
+          <t>GRE LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="AE77" t="inlineStr">
+        <is>
+          <t>UGEL SÁNCHEZ CARRIÓN</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -8477,6 +9247,16 @@
           <t>130107</t>
         </is>
       </c>
+      <c r="AD78" t="inlineStr">
+        <is>
+          <t>GRE LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="AE78" t="inlineStr">
+        <is>
+          <t>UGEL 04 - TRUJILLO SUR ESTE</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -8594,6 +9374,16 @@
           <t>130107</t>
         </is>
       </c>
+      <c r="AD79" t="inlineStr">
+        <is>
+          <t>GRE LA LIBERTAD</t>
+        </is>
+      </c>
+      <c r="AE79" t="inlineStr">
+        <is>
+          <t>UGEL 04 - TRUJILLO SUR ESTE</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -8705,6 +9495,16 @@
       <c r="AC80" t="inlineStr">
         <is>
           <t>140303</t>
+        </is>
+      </c>
+      <c r="AD80" t="inlineStr">
+        <is>
+          <t>GRE LAMBAYEQUE</t>
+        </is>
+      </c>
+      <c r="AE80" t="inlineStr">
+        <is>
+          <t>UGEL LAMBAYEQUE</t>
         </is>
       </c>
     </row>
@@ -8810,6 +9610,16 @@
           <t>150601</t>
         </is>
       </c>
+      <c r="AD81" t="inlineStr">
+        <is>
+          <t>DRE LIMA PROVINCIAS</t>
+        </is>
+      </c>
+      <c r="AE81" t="inlineStr">
+        <is>
+          <t>UGEL 10 HUARAL</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -8919,6 +9729,16 @@
           <t>150601</t>
         </is>
       </c>
+      <c r="AD82" t="inlineStr">
+        <is>
+          <t>DRE LIMA PROVINCIAS</t>
+        </is>
+      </c>
+      <c r="AE82" t="inlineStr">
+        <is>
+          <t>UGEL 10 HUARAL</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -9028,6 +9848,16 @@
           <t>150601</t>
         </is>
       </c>
+      <c r="AD83" t="inlineStr">
+        <is>
+          <t>DRE LIMA PROVINCIAS</t>
+        </is>
+      </c>
+      <c r="AE83" t="inlineStr">
+        <is>
+          <t>UGEL 10 HUARAL</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -9135,6 +9965,16 @@
       <c r="AC84" t="inlineStr">
         <is>
           <t>150601</t>
+        </is>
+      </c>
+      <c r="AD84" t="inlineStr">
+        <is>
+          <t>DRE LIMA PROVINCIAS</t>
+        </is>
+      </c>
+      <c r="AE84" t="inlineStr">
+        <is>
+          <t>UGEL 10 HUARAL</t>
         </is>
       </c>
     </row>
@@ -9230,6 +10070,16 @@
           <t>150203</t>
         </is>
       </c>
+      <c r="AD85" t="inlineStr">
+        <is>
+          <t>DRE LIMA PROVINCIAS</t>
+        </is>
+      </c>
+      <c r="AE85" t="inlineStr">
+        <is>
+          <t>UGEL 16 BARRANCA</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -9345,6 +10195,16 @@
           <t>160510</t>
         </is>
       </c>
+      <c r="AD86" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE86" t="inlineStr">
+        <is>
+          <t>UGEL REQUENA</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -9460,6 +10320,16 @@
           <t>160510</t>
         </is>
       </c>
+      <c r="AD87" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE87" t="inlineStr">
+        <is>
+          <t>UGEL REQUENA</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -9575,6 +10445,16 @@
           <t>160510</t>
         </is>
       </c>
+      <c r="AD88" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE88" t="inlineStr">
+        <is>
+          <t>UGEL REQUENA</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -9688,6 +10568,16 @@
       <c r="AC89" t="inlineStr">
         <is>
           <t>160510</t>
+        </is>
+      </c>
+      <c r="AD89" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE89" t="inlineStr">
+        <is>
+          <t>UGEL REQUENA</t>
         </is>
       </c>
     </row>
@@ -9785,6 +10675,16 @@
           <t>160604</t>
         </is>
       </c>
+      <c r="AD90" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE90" t="inlineStr">
+        <is>
+          <t>UGEL UCAYALI-CONTAMANA</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -9902,6 +10802,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD91" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE91" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -10019,6 +10929,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD92" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE92" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -10136,6 +11056,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD93" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE93" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -10253,6 +11183,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE94" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -10370,6 +11310,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE95" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -10487,6 +11437,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE96" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -10604,6 +11564,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE97" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -10721,6 +11691,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE98" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -10838,6 +11818,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE99" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -10955,6 +11945,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD100" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE100" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -11072,6 +12072,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD101" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE101" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -11189,6 +12199,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD102" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE102" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -11306,6 +12326,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD103" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE103" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -11423,6 +12453,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD104" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE104" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11540,6 +12580,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD105" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE105" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -11657,6 +12707,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD106" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE106" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -11774,6 +12834,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD107" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE107" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -11891,6 +12961,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD108" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE108" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -12008,6 +13088,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD109" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE109" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -12125,6 +13215,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD110" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE110" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -12242,6 +13342,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD111" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE111" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -12359,6 +13469,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD112" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE112" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -12476,6 +13596,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD113" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE113" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -12593,6 +13723,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD114" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE114" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -12710,6 +13850,16 @@
           <t>160210</t>
         </is>
       </c>
+      <c r="AD115" t="inlineStr">
+        <is>
+          <t>DRE LORETO</t>
+        </is>
+      </c>
+      <c r="AE115" t="inlineStr">
+        <is>
+          <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -12811,6 +13961,16 @@
           <t>170202</t>
         </is>
       </c>
+      <c r="AD116" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE116" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -12916,6 +14076,16 @@
           <t>170202</t>
         </is>
       </c>
+      <c r="AD117" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE117" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -13021,6 +14191,16 @@
           <t>170202</t>
         </is>
       </c>
+      <c r="AD118" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE118" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -13126,6 +14306,16 @@
           <t>170202</t>
         </is>
       </c>
+      <c r="AD119" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE119" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -13231,6 +14421,16 @@
           <t>170202</t>
         </is>
       </c>
+      <c r="AD120" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE120" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -13336,6 +14536,16 @@
           <t>170202</t>
         </is>
       </c>
+      <c r="AD121" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE121" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -13433,6 +14643,16 @@
           <t>170202</t>
         </is>
       </c>
+      <c r="AD122" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE122" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -13538,6 +14758,16 @@
           <t>170202</t>
         </is>
       </c>
+      <c r="AD123" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE123" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -13643,6 +14873,16 @@
           <t>170204</t>
         </is>
       </c>
+      <c r="AD124" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE124" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -13740,6 +14980,16 @@
           <t>170204</t>
         </is>
       </c>
+      <c r="AD125" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE125" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -13845,6 +15095,16 @@
           <t>170204</t>
         </is>
       </c>
+      <c r="AD126" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE126" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -13942,6 +15202,16 @@
           <t>170204</t>
         </is>
       </c>
+      <c r="AD127" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE127" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -14039,6 +15309,16 @@
           <t>170302</t>
         </is>
       </c>
+      <c r="AD128" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE128" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -14136,6 +15416,16 @@
           <t>170302</t>
         </is>
       </c>
+      <c r="AD129" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE129" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -14233,6 +15523,16 @@
           <t>170302</t>
         </is>
       </c>
+      <c r="AD130" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE130" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -14338,6 +15638,16 @@
           <t>170302</t>
         </is>
       </c>
+      <c r="AD131" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE131" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -14443,6 +15753,16 @@
           <t>170302</t>
         </is>
       </c>
+      <c r="AD132" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE132" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -14548,6 +15868,16 @@
           <t>170302</t>
         </is>
       </c>
+      <c r="AD133" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE133" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -14649,6 +15979,16 @@
           <t>170302</t>
         </is>
       </c>
+      <c r="AD134" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE134" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -14746,6 +16086,16 @@
           <t>170302</t>
         </is>
       </c>
+      <c r="AD135" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE135" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -14847,6 +16197,16 @@
           <t>170102</t>
         </is>
       </c>
+      <c r="AD136" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE136" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -14948,6 +16308,16 @@
           <t>170102</t>
         </is>
       </c>
+      <c r="AD137" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE137" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -15049,6 +16419,16 @@
           <t>170102</t>
         </is>
       </c>
+      <c r="AD138" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE138" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -15154,6 +16534,16 @@
           <t>170102</t>
         </is>
       </c>
+      <c r="AD139" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE139" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -15255,6 +16645,16 @@
           <t>170102</t>
         </is>
       </c>
+      <c r="AD140" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE140" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -15360,6 +16760,16 @@
           <t>170102</t>
         </is>
       </c>
+      <c r="AD141" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE141" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -15465,6 +16875,16 @@
           <t>170102</t>
         </is>
       </c>
+      <c r="AD142" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE142" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -15566,6 +16986,16 @@
           <t>170102</t>
         </is>
       </c>
+      <c r="AD143" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE143" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -15671,6 +17101,16 @@
           <t>170301</t>
         </is>
       </c>
+      <c r="AD144" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE144" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -15776,6 +17216,16 @@
           <t>170301</t>
         </is>
       </c>
+      <c r="AD145" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE145" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -15881,6 +17331,16 @@
           <t>170301</t>
         </is>
       </c>
+      <c r="AD146" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE146" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -15986,6 +17446,16 @@
           <t>170104</t>
         </is>
       </c>
+      <c r="AD147" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE147" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -16091,6 +17561,16 @@
           <t>170104</t>
         </is>
       </c>
+      <c r="AD148" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE148" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -16188,6 +17668,16 @@
           <t>170104</t>
         </is>
       </c>
+      <c r="AD149" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE149" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -16293,6 +17783,16 @@
           <t>170104</t>
         </is>
       </c>
+      <c r="AD150" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE150" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -16398,6 +17898,16 @@
           <t>170104</t>
         </is>
       </c>
+      <c r="AD151" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE151" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -16503,6 +18013,16 @@
           <t>170104</t>
         </is>
       </c>
+      <c r="AD152" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE152" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -16608,6 +18128,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD153" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE153" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -16705,6 +18235,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD154" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE154" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -16810,6 +18350,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD155" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE155" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -16915,6 +18465,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD156" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE156" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -17020,6 +18580,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD157" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE157" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -17125,6 +18695,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD158" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE158" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -17230,6 +18810,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD159" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE159" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -17327,6 +18917,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD160" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE160" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -17428,6 +19028,16 @@
           <t>170103</t>
         </is>
       </c>
+      <c r="AD161" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE161" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -17533,6 +19143,16 @@
           <t>170203</t>
         </is>
       </c>
+      <c r="AD162" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE162" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -17638,6 +19258,16 @@
           <t>170203</t>
         </is>
       </c>
+      <c r="AD163" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE163" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -17743,6 +19373,16 @@
           <t>170203</t>
         </is>
       </c>
+      <c r="AD164" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE164" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -17840,6 +19480,16 @@
           <t>170203</t>
         </is>
       </c>
+      <c r="AD165" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE165" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -17945,6 +19595,16 @@
           <t>170203</t>
         </is>
       </c>
+      <c r="AD166" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE166" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -18050,6 +19710,16 @@
           <t>170203</t>
         </is>
       </c>
+      <c r="AD167" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE167" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -18147,6 +19817,16 @@
           <t>170201</t>
         </is>
       </c>
+      <c r="AD168" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE168" t="inlineStr">
+        <is>
+          <t>UGEL MANU</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -18252,6 +19932,16 @@
           <t>170303</t>
         </is>
       </c>
+      <c r="AD169" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE169" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -18349,6 +20039,16 @@
           <t>170303</t>
         </is>
       </c>
+      <c r="AD170" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE170" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -18446,6 +20146,16 @@
           <t>170303</t>
         </is>
       </c>
+      <c r="AD171" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE171" t="inlineStr">
+        <is>
+          <t>UGEL TAHUAMANU</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -18551,6 +20261,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD172" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE172" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -18656,6 +20376,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD173" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE173" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -18761,6 +20491,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD174" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE174" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -18866,6 +20606,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD175" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE175" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -18971,6 +20721,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD176" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE176" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -19076,6 +20836,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD177" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE177" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -19173,6 +20943,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD178" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE178" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -19278,6 +21058,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD179" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE179" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -19383,6 +21173,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD180" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE180" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -19488,6 +21288,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD181" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE181" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -19593,6 +21403,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD182" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE182" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -19698,6 +21518,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD183" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE183" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -19795,6 +21625,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD184" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE184" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -19900,6 +21740,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD185" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE185" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -20005,6 +21855,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD186" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE186" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -20110,6 +21970,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD187" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE187" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -20215,6 +22085,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD188" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE188" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -20312,6 +22192,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD189" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE189" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -20417,6 +22307,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD190" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE190" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -20522,6 +22422,16 @@
           <t>170101</t>
         </is>
       </c>
+      <c r="AD191" t="inlineStr">
+        <is>
+          <t>DRE MADRE DE DIOS</t>
+        </is>
+      </c>
+      <c r="AE191" t="inlineStr">
+        <is>
+          <t>UGEL TAMBOPATA</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -20639,6 +22549,16 @@
           <t>200606</t>
         </is>
       </c>
+      <c r="AD192" t="inlineStr">
+        <is>
+          <t>DRE PIURA</t>
+        </is>
+      </c>
+      <c r="AE192" t="inlineStr">
+        <is>
+          <t>UGEL SULLANA</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -20738,6 +22658,16 @@
       <c r="AC193" t="inlineStr">
         <is>
           <t>220806</t>
+        </is>
+      </c>
+      <c r="AD193" t="inlineStr">
+        <is>
+          <t>DRE SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="AE193" t="inlineStr">
+        <is>
+          <t>UGEL RIOJA</t>
         </is>
       </c>
     </row>
@@ -20833,6 +22763,16 @@
           <t>220806</t>
         </is>
       </c>
+      <c r="AD194" t="inlineStr">
+        <is>
+          <t>DRE SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="AE194" t="inlineStr">
+        <is>
+          <t>UGEL RIOJA</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -20922,6 +22862,16 @@
           <t>220808</t>
         </is>
       </c>
+      <c r="AD195" t="inlineStr">
+        <is>
+          <t>DRE SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="AE195" t="inlineStr">
+        <is>
+          <t>UGEL RIOJA</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -21011,6 +22961,16 @@
           <t>220808</t>
         </is>
       </c>
+      <c r="AD196" t="inlineStr">
+        <is>
+          <t>DRE SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="AE196" t="inlineStr">
+        <is>
+          <t>UGEL RIOJA</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -21100,6 +23060,16 @@
           <t>220808</t>
         </is>
       </c>
+      <c r="AD197" t="inlineStr">
+        <is>
+          <t>DRE SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="AE197" t="inlineStr">
+        <is>
+          <t>UGEL RIOJA</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -21189,6 +23159,16 @@
           <t>220808</t>
         </is>
       </c>
+      <c r="AD198" t="inlineStr">
+        <is>
+          <t>DRE SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="AE198" t="inlineStr">
+        <is>
+          <t>UGEL RIOJA</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -21278,6 +23258,16 @@
           <t>220808</t>
         </is>
       </c>
+      <c r="AD199" t="inlineStr">
+        <is>
+          <t>DRE SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="AE199" t="inlineStr">
+        <is>
+          <t>UGEL RIOJA</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -21365,6 +23355,16 @@
       <c r="AC200" t="inlineStr">
         <is>
           <t>220808</t>
+        </is>
+      </c>
+      <c r="AD200" t="inlineStr">
+        <is>
+          <t>DRE SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="AE200" t="inlineStr">
+        <is>
+          <t>UGEL RIOJA</t>
         </is>
       </c>
     </row>
@@ -21460,6 +23460,16 @@
           <t>230105</t>
         </is>
       </c>
+      <c r="AD201" t="inlineStr">
+        <is>
+          <t>DRE TACNA</t>
+        </is>
+      </c>
+      <c r="AE201" t="inlineStr">
+        <is>
+          <t>UGEL TACNA</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -21551,6 +23561,16 @@
       <c r="AC202" t="inlineStr">
         <is>
           <t>230105</t>
+        </is>
+      </c>
+      <c r="AD202" t="inlineStr">
+        <is>
+          <t>DRE TACNA</t>
+        </is>
+      </c>
+      <c r="AE202" t="inlineStr">
+        <is>
+          <t>UGEL TACNA</t>
         </is>
       </c>
     </row>
@@ -21642,6 +23662,16 @@
           <t>230105</t>
         </is>
       </c>
+      <c r="AD203" t="inlineStr">
+        <is>
+          <t>DRE TACNA</t>
+        </is>
+      </c>
+      <c r="AE203" t="inlineStr">
+        <is>
+          <t>UGEL TACNA</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -21731,6 +23761,16 @@
           <t>230105</t>
         </is>
       </c>
+      <c r="AD204" t="inlineStr">
+        <is>
+          <t>DRE TACNA</t>
+        </is>
+      </c>
+      <c r="AE204" t="inlineStr">
+        <is>
+          <t>UGEL TACNA</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -21820,6 +23860,16 @@
           <t>230105</t>
         </is>
       </c>
+      <c r="AD205" t="inlineStr">
+        <is>
+          <t>DRE TACNA</t>
+        </is>
+      </c>
+      <c r="AE205" t="inlineStr">
+        <is>
+          <t>UGEL TACNA</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -21909,6 +23959,16 @@
           <t>230105</t>
         </is>
       </c>
+      <c r="AD206" t="inlineStr">
+        <is>
+          <t>DRE TACNA</t>
+        </is>
+      </c>
+      <c r="AE206" t="inlineStr">
+        <is>
+          <t>UGEL TACNA</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -21996,6 +24056,16 @@
           <t>230101</t>
         </is>
       </c>
+      <c r="AD207" t="inlineStr">
+        <is>
+          <t>DRE TACNA</t>
+        </is>
+      </c>
+      <c r="AE207" t="inlineStr">
+        <is>
+          <t>UGEL TACNA</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Integra padron web, campo fuente y Grupo 2 final (df_pi_listados_final_v7)
- Padron web nacional (Copia de Padron_web.csv) como insumo adicional: amplia
  imputacion de cod_local (cod_mod/codinst) y respaldo geografico. cod_local
  sube a 99.8% y geografia/UGEL a 99.6%.
- Nuevo campo 'fuente' en todas las bases (unidad que reporta); en Anexo 1 y 2
  se toma por fila del campo Remitente.
- Incorpora el Grupo 2 (PI) con su base final ya limpia df_pi_listados_final_v7
  (hoja con_cod_local), estandarizando codigos, fechas, montos, ubigeo y fuente.
- Base final armonizada ahora cubre los 11 grupos (337,120 filas).

https://claude.ai/code/session_01N9afypBcQVKYhttom8P34Z
</commit_message>
<xml_diff>
--- a/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_anexo2_b.xlsx
+++ b/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_anexo2_b.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE207"/>
+  <dimension ref="A1:AF207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,6 +576,11 @@
           <t>ugel</t>
         </is>
       </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>fuente</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -699,6 +704,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -822,6 +832,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -943,6 +958,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1066,6 +1086,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1189,6 +1214,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1314,6 +1344,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1437,6 +1472,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1560,6 +1600,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1683,6 +1728,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1806,6 +1856,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1929,6 +1984,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2048,6 +2108,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2169,6 +2234,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2292,6 +2362,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2421,6 +2496,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2542,6 +2622,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2665,6 +2750,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2790,6 +2880,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2911,6 +3006,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3034,6 +3134,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3157,6 +3262,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3280,6 +3390,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3403,6 +3518,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3526,6 +3646,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3649,6 +3774,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3772,6 +3902,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3895,6 +4030,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -4018,6 +4158,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4143,6 +4288,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4264,6 +4414,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4387,6 +4542,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -4510,6 +4670,11 @@
           <t>UGEL BAGUA</t>
         </is>
       </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4631,6 +4796,11 @@
       <c r="AE34" t="inlineStr">
         <is>
           <t>UGEL BAGUA</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
     </row>
@@ -4738,6 +4908,11 @@
       <c r="AE35" t="inlineStr">
         <is>
           <t>UGEL CHACHAPOYAS</t>
+        </is>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Levanto</t>
         </is>
       </c>
     </row>
@@ -4837,6 +5012,11 @@
           <t>UGEL HUARI</t>
         </is>
       </c>
+      <c r="AF36" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Huari</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -4950,6 +5130,11 @@
           <t>UGEL POMABAMBA</t>
         </is>
       </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Quinuabamba</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -5067,6 +5252,11 @@
           <t>UGEL CHINCHEROS</t>
         </is>
       </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Cochcarcas</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -5184,6 +5374,11 @@
           <t>UGEL CHINCHEROS</t>
         </is>
       </c>
+      <c r="AF39" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Cochcarcas</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -5303,6 +5498,11 @@
           <t>UGEL CHINCHEROS</t>
         </is>
       </c>
+      <c r="AF40" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Cochcarcas</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -5420,6 +5620,11 @@
           <t>UGEL CHINCHEROS</t>
         </is>
       </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Cochcarcas</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -5539,6 +5744,11 @@
           <t>UGEL CHINCHEROS</t>
         </is>
       </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Cochcarcas</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -5654,6 +5864,11 @@
       <c r="AE43" t="inlineStr">
         <is>
           <t>UGEL CHINCHEROS</t>
+        </is>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Cochcarcas</t>
         </is>
       </c>
     </row>
@@ -5761,6 +5976,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -5866,6 +6086,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -5971,6 +6196,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -6076,6 +6306,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF47" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -6181,6 +6416,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF48" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -6286,6 +6526,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF49" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -6391,6 +6636,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF50" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -6496,6 +6746,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF51" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -6601,6 +6856,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -6706,6 +6966,11 @@
           <t>UGEL CARAVELI</t>
         </is>
       </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Acari</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -6831,6 +7096,11 @@
       <c r="AE54" t="inlineStr">
         <is>
           <t>UGEL CANGALLO</t>
+        </is>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Cangallo</t>
         </is>
       </c>
     </row>
@@ -6934,6 +7204,11 @@
           <t>UGEL LUCANAS</t>
         </is>
       </c>
+      <c r="AF55" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Carmen Salcedo</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -7033,6 +7308,11 @@
       <c r="AE56" t="inlineStr">
         <is>
           <t>UGEL LUCANAS</t>
+        </is>
+      </c>
+      <c r="AF56" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Carmen Salcedo</t>
         </is>
       </c>
     </row>
@@ -7128,6 +7408,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -7221,6 +7506,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -7314,6 +7604,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF59" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -7407,6 +7702,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF60" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -7500,6 +7800,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF61" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -7593,6 +7898,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF62" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -7686,6 +7996,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF63" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -7779,6 +8094,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF64" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -7872,6 +8192,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -7965,6 +8290,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF66" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -8058,6 +8388,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF67" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -8151,6 +8486,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF68" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -8244,6 +8584,11 @@
           <t>UGEL LA MAR</t>
         </is>
       </c>
+      <c r="AF69" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Chilcas</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -8347,6 +8692,11 @@
           <t>UGEL VENTANILLA</t>
         </is>
       </c>
+      <c r="AF70" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Mi Peru</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -8464,6 +8814,11 @@
           <t>UGEL VENTANILLA</t>
         </is>
       </c>
+      <c r="AF71" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Mi Peru</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -8573,6 +8928,11 @@
       <c r="AE72" t="inlineStr">
         <is>
           <t>UGEL VENTANILLA</t>
+        </is>
+      </c>
+      <c r="AF72" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Mi Peru</t>
         </is>
       </c>
     </row>
@@ -8682,6 +9042,11 @@
           <t>UGEL VENTANILLA</t>
         </is>
       </c>
+      <c r="AF73" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Mi Peru</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -8795,6 +9160,11 @@
           <t>UGEL HUÁNUCO</t>
         </is>
       </c>
+      <c r="AF74" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Maria del Valle</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -8902,6 +9272,11 @@
           <t>UGEL SÁNCHEZ CARRIÓN</t>
         </is>
       </c>
+      <c r="AF75" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Marcabal</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -9033,6 +9408,11 @@
       <c r="AE76" t="inlineStr">
         <is>
           <t>UGEL SÁNCHEZ CARRIÓN</t>
+        </is>
+      </c>
+      <c r="AF76" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Marcabal</t>
         </is>
       </c>
     </row>
@@ -9138,6 +9518,11 @@
           <t>UGEL SÁNCHEZ CARRIÓN</t>
         </is>
       </c>
+      <c r="AF77" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Marcabal</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -9257,6 +9642,11 @@
           <t>UGEL 04 - TRUJILLO SUR ESTE</t>
         </is>
       </c>
+      <c r="AF78" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Moche</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -9384,6 +9774,11 @@
           <t>UGEL 04 - TRUJILLO SUR ESTE</t>
         </is>
       </c>
+      <c r="AF79" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Moche</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -9505,6 +9900,11 @@
       <c r="AE80" t="inlineStr">
         <is>
           <t>UGEL LAMBAYEQUE</t>
+        </is>
+      </c>
+      <c r="AF80" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Illimo</t>
         </is>
       </c>
     </row>
@@ -9620,6 +10020,11 @@
           <t>UGEL 10 HUARAL</t>
         </is>
       </c>
+      <c r="AF81" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Huaral</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -9739,6 +10144,11 @@
           <t>UGEL 10 HUARAL</t>
         </is>
       </c>
+      <c r="AF82" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Huaral</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -9858,6 +10268,11 @@
           <t>UGEL 10 HUARAL</t>
         </is>
       </c>
+      <c r="AF83" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Huaral</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -9975,6 +10390,11 @@
       <c r="AE84" t="inlineStr">
         <is>
           <t>UGEL 10 HUARAL</t>
+        </is>
+      </c>
+      <c r="AF84" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Huaral</t>
         </is>
       </c>
     </row>
@@ -10080,6 +10500,11 @@
           <t>UGEL 16 BARRANCA</t>
         </is>
       </c>
+      <c r="AF85" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Pativilca</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -10205,6 +10630,11 @@
           <t>UGEL REQUENA</t>
         </is>
       </c>
+      <c r="AF86" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Jenaro Herrera</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -10330,6 +10760,11 @@
           <t>UGEL REQUENA</t>
         </is>
       </c>
+      <c r="AF87" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Jenaro Herrera</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -10455,6 +10890,11 @@
           <t>UGEL REQUENA</t>
         </is>
       </c>
+      <c r="AF88" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Jenaro Herrera</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -10578,6 +11018,11 @@
       <c r="AE89" t="inlineStr">
         <is>
           <t>UGEL REQUENA</t>
+        </is>
+      </c>
+      <c r="AF89" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Jenaro Herrera</t>
         </is>
       </c>
     </row>
@@ -10685,6 +11130,11 @@
           <t>UGEL UCAYALI-CONTAMANA</t>
         </is>
       </c>
+      <c r="AF90" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Pampa Hermosa</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -10812,6 +11262,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF91" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -10939,6 +11394,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF92" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -11066,6 +11526,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF93" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -11193,6 +11658,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF94" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -11320,6 +11790,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF95" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -11447,6 +11922,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -11574,6 +12054,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF97" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -11701,6 +12186,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF98" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -11828,6 +12318,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF99" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -11955,6 +12450,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF100" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -12082,6 +12582,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF101" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -12209,6 +12714,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF102" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -12336,6 +12846,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF103" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -12463,6 +12978,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF104" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -12590,6 +13110,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF105" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -12717,6 +13242,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF106" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -12844,6 +13374,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF107" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -12971,6 +13506,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF108" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -13098,6 +13638,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF109" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -13225,6 +13770,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF110" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -13352,6 +13902,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF111" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -13479,6 +14034,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF112" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -13606,6 +14166,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF113" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -13733,6 +14298,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF114" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -13860,6 +14430,11 @@
           <t>UGEL ALTO AMAZONAS-YURIMAGUAS</t>
         </is>
       </c>
+      <c r="AF115" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Santa Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -13971,6 +14546,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF116" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -14086,6 +14666,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF117" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -14201,6 +14786,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF118" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -14316,6 +14906,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF119" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -14431,6 +15026,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF120" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -14546,6 +15146,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF121" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -14653,6 +15258,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF122" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -14768,6 +15378,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF123" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -14883,6 +15498,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF124" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -14990,6 +15610,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF125" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -15105,6 +15730,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF126" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -15212,6 +15842,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF127" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -15319,6 +15954,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF128" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -15426,6 +16066,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -15533,6 +16178,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF130" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -15648,6 +16298,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF131" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -15763,6 +16418,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF132" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -15878,6 +16538,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF133" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -15989,6 +16654,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF134" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -16096,6 +16766,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF135" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -16207,6 +16882,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF136" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -16318,6 +16998,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF137" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -16429,6 +17114,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF138" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -16544,6 +17234,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF139" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -16655,6 +17350,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF140" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -16770,6 +17470,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF141" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -16885,6 +17590,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF142" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -16996,6 +17706,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF143" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -17111,6 +17826,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF144" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -17226,6 +17946,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF145" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -17341,6 +18066,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF146" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -17456,6 +18186,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF147" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -17571,6 +18306,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF148" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -17678,6 +18418,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF149" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -17793,6 +18538,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF150" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -17908,6 +18658,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF151" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -18023,6 +18778,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF152" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -18138,6 +18898,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF153" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -18245,6 +19010,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF154" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -18360,6 +19130,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF155" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -18475,6 +19250,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF156" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -18590,6 +19370,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF157" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -18705,6 +19490,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF158" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -18820,6 +19610,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF159" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -18927,6 +19722,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF160" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -19038,6 +19838,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF161" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -19153,6 +19958,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF162" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -19268,6 +20078,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF163" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -19383,6 +20198,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF164" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -19490,6 +20310,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF165" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -19605,6 +20430,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF166" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -19720,6 +20550,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF167" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -19827,6 +20662,11 @@
           <t>UGEL MANU</t>
         </is>
       </c>
+      <c r="AF168" t="inlineStr">
+        <is>
+          <t>Anexo 2 - GORE Madre de Dios</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -19942,6 +20782,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF169" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Tahuamanu</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -20049,6 +20894,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF170" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Tahuamanu</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -20156,6 +21006,11 @@
           <t>UGEL TAHUAMANU</t>
         </is>
       </c>
+      <c r="AF171" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Tahuamanu</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -20271,6 +21126,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF172" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -20386,6 +21246,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF173" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -20501,6 +21366,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF174" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -20616,6 +21486,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF175" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -20731,6 +21606,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF176" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -20846,6 +21726,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF177" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -20953,6 +21838,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF178" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -21068,6 +21958,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF179" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -21183,6 +22078,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF180" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -21298,6 +22198,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF181" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -21413,6 +22318,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF182" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -21528,6 +22438,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF183" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -21635,6 +22550,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF184" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -21750,6 +22670,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF185" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -21865,6 +22790,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF186" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -21980,6 +22910,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF187" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -22095,6 +23030,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF188" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -22202,6 +23142,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF189" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -22317,6 +23262,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF190" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -22432,6 +23382,11 @@
           <t>UGEL TAMBOPATA</t>
         </is>
       </c>
+      <c r="AF191" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tambopata</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -22559,6 +23514,11 @@
           <t>UGEL SULLANA</t>
         </is>
       </c>
+      <c r="AF192" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Sullana</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -22668,6 +23628,11 @@
       <c r="AE193" t="inlineStr">
         <is>
           <t>UGEL RIOJA</t>
+        </is>
+      </c>
+      <c r="AF193" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Posic</t>
         </is>
       </c>
     </row>
@@ -22773,6 +23738,11 @@
           <t>UGEL RIOJA</t>
         </is>
       </c>
+      <c r="AF194" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Posic</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -22872,6 +23842,11 @@
           <t>UGEL RIOJA</t>
         </is>
       </c>
+      <c r="AF195" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Yorongos</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -22971,6 +23946,11 @@
           <t>UGEL RIOJA</t>
         </is>
       </c>
+      <c r="AF196" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Yorongos</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -23070,6 +24050,11 @@
           <t>UGEL RIOJA</t>
         </is>
       </c>
+      <c r="AF197" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Yorongos</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -23169,6 +24154,11 @@
           <t>UGEL RIOJA</t>
         </is>
       </c>
+      <c r="AF198" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Yorongos</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -23268,6 +24258,11 @@
           <t>UGEL RIOJA</t>
         </is>
       </c>
+      <c r="AF199" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Yorongos</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -23365,6 +24360,11 @@
       <c r="AE200" t="inlineStr">
         <is>
           <t>UGEL RIOJA</t>
+        </is>
+      </c>
+      <c r="AF200" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MD Yorongos</t>
         </is>
       </c>
     </row>
@@ -23470,6 +24470,11 @@
           <t>UGEL TACNA</t>
         </is>
       </c>
+      <c r="AF201" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tacna</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -23571,6 +24576,11 @@
       <c r="AE202" t="inlineStr">
         <is>
           <t>UGEL TACNA</t>
+        </is>
+      </c>
+      <c r="AF202" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tacna</t>
         </is>
       </c>
     </row>
@@ -23672,6 +24682,11 @@
           <t>UGEL TACNA</t>
         </is>
       </c>
+      <c r="AF203" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tacna</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -23771,6 +24786,11 @@
           <t>UGEL TACNA</t>
         </is>
       </c>
+      <c r="AF204" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tacna</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -23870,6 +24890,11 @@
           <t>UGEL TACNA</t>
         </is>
       </c>
+      <c r="AF205" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tacna</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -23969,6 +24994,11 @@
           <t>UGEL TACNA</t>
         </is>
       </c>
+      <c r="AF206" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tacna</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -24066,6 +25096,11 @@
           <t>UGEL TACNA</t>
         </is>
       </c>
+      <c r="AF207" t="inlineStr">
+        <is>
+          <t>Anexo 2 - MP Tacna</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Agrega nombre de institucion, ambito urbano/rural y cruce geografico por nombre
- Nueva columna nombre_ie (nombre de la institucion educativa) en todas las
  bases, derivada del padron/ubigeo por cod_local (cobertura 97.6%).
- Nueva columna area (ambito Urbano/Rural) desde el padron web (99.6%).
- Para registros sin cod_local, asigna departamento/DRE/UGEL cruzando por
  nombre de Unidad Zonal o UGEL contra el padron (df_uz_asesoramiento pasa de
  0 a 650/651 con departamento).
- Cobertura final: departamento/DRE 99.9%, UGEL 99.7%.

https://claude.ai/code/session_01N9afypBcQVKYhttom8P34Z
</commit_message>
<xml_diff>
--- a/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_anexo2_b.xlsx
+++ b/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_anexo2_b.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF207"/>
+  <dimension ref="A1:AH207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -578,6 +578,16 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>nombre_ie</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
           <t>fuente</t>
         </is>
       </c>
@@ -706,6 +716,16 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
+          <t>262</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -834,6 +854,16 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
+          <t>16199</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -960,6 +990,16 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
+          <t>16200</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -1088,6 +1128,16 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
+          <t>16201</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -1216,6 +1266,16 @@
       </c>
       <c r="AF6" t="inlineStr">
         <is>
+          <t>16203</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -1346,6 +1406,16 @@
       </c>
       <c r="AF7" t="inlineStr">
         <is>
+          <t>16207</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -1474,6 +1544,16 @@
       </c>
       <c r="AF8" t="inlineStr">
         <is>
+          <t>16591</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -1602,6 +1682,16 @@
       </c>
       <c r="AF9" t="inlineStr">
         <is>
+          <t>16605 JESUS DE NAZARETH/16605 JESUS DE NAZARETH</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -1730,6 +1820,16 @@
       </c>
       <c r="AF10" t="inlineStr">
         <is>
+          <t>16205</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -1858,6 +1958,16 @@
       </c>
       <c r="AF11" t="inlineStr">
         <is>
+          <t>16206/16206</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -1986,6 +2096,16 @@
       </c>
       <c r="AF12" t="inlineStr">
         <is>
+          <t>AMAZONAS</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -2110,6 +2230,16 @@
       </c>
       <c r="AF13" t="inlineStr">
         <is>
+          <t>16194/16194/16194</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -2236,6 +2366,16 @@
       </c>
       <c r="AF14" t="inlineStr">
         <is>
+          <t>16192/16192/16192</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -2364,6 +2504,16 @@
       </c>
       <c r="AF15" t="inlineStr">
         <is>
+          <t>16193/16193</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -2498,6 +2648,16 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
+          <t>16989</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -2624,6 +2784,16 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
+          <t>17300</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -2752,6 +2922,16 @@
       </c>
       <c r="AF18" t="inlineStr">
         <is>
+          <t>LA INMACULADA/LA INMACULADA/LA INMACULADA</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -2882,6 +3062,16 @@
       </c>
       <c r="AF19" t="inlineStr">
         <is>
+          <t>AGROPECUARIO TORIBIO RODRIGUEZ DE MENDOZA/AGROPECUARIO TORIBIO RODRIGUEZ DE MENDOZA/AGROPECUARIO TORIBIO RODRIGUEZ DE MENDOZA</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -3008,6 +3198,16 @@
       </c>
       <c r="AF20" t="inlineStr">
         <is>
+          <t>TECNICO INDUSTRIAL BAGUA</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -3136,6 +3336,16 @@
       </c>
       <c r="AF21" t="inlineStr">
         <is>
+          <t>001/001</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -3264,6 +3474,16 @@
       </c>
       <c r="AF22" t="inlineStr">
         <is>
+          <t>16239/16239</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -3392,6 +3612,16 @@
       </c>
       <c r="AF23" t="inlineStr">
         <is>
+          <t>SAGRADO CORAZON</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -3520,6 +3750,16 @@
       </c>
       <c r="AF24" t="inlineStr">
         <is>
+          <t>219</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -3648,6 +3888,16 @@
       </c>
       <c r="AF25" t="inlineStr">
         <is>
+          <t>DIVINO MAESTRO</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -3776,6 +4026,16 @@
       </c>
       <c r="AF26" t="inlineStr">
         <is>
+          <t>273</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -3904,6 +4164,16 @@
       </c>
       <c r="AF27" t="inlineStr">
         <is>
+          <t>16195</t>
+        </is>
+      </c>
+      <c r="AG27" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -4032,6 +4302,16 @@
       </c>
       <c r="AF28" t="inlineStr">
         <is>
+          <t>16275/16275</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -4160,6 +4440,16 @@
       </c>
       <c r="AF29" t="inlineStr">
         <is>
+          <t>16752</t>
+        </is>
+      </c>
+      <c r="AG29" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -4290,6 +4580,16 @@
       </c>
       <c r="AF30" t="inlineStr">
         <is>
+          <t>16277/16277</t>
+        </is>
+      </c>
+      <c r="AG30" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -4416,6 +4716,16 @@
       </c>
       <c r="AF31" t="inlineStr">
         <is>
+          <t>16283/16283/16283</t>
+        </is>
+      </c>
+      <c r="AG31" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -4544,6 +4854,16 @@
       </c>
       <c r="AF32" t="inlineStr">
         <is>
+          <t>JOSE CARLOS MARIATEGUI/JOSE CARLOS MARIATEGUI/JOSE CARLOS MARIATEGUI</t>
+        </is>
+      </c>
+      <c r="AG32" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -4672,6 +4992,16 @@
       </c>
       <c r="AF33" t="inlineStr">
         <is>
+          <t>MANUEL SCORZA</t>
+        </is>
+      </c>
+      <c r="AG33" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
       </c>
@@ -4799,6 +5129,16 @@
         </is>
       </c>
       <c r="AF34" t="inlineStr">
+        <is>
+          <t>NUESTRA SEÑORA DE GUADALUPE FE Y ALEGRIA 31/NUESTRA SEÑORA DE GUADALUPE FE Y ALEGRIA 31/NUESTRA SEÑORA DE GUADALUPE FE Y ALEGRIA 31/NUESTRA SEÑORA DE GUADALUPE FE Y ALEGRIA 31/NUESTRA SEÑORA DE GUADALUPE FE Y ALEGRIA 31</t>
+        </is>
+      </c>
+      <c r="AG34" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH34" t="inlineStr">
         <is>
           <t>Anexo 2 - GORE Amazonas</t>
         </is>
@@ -4911,6 +5251,16 @@
         </is>
       </c>
       <c r="AF35" t="inlineStr">
+        <is>
+          <t>18052 PADRE BLAS VALERA PEREZ/18052 PADRE BLAS VALERA PEREZ</t>
+        </is>
+      </c>
+      <c r="AG35" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH35" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Levanto</t>
         </is>
@@ -5014,6 +5364,16 @@
       </c>
       <c r="AF36" t="inlineStr">
         <is>
+          <t>VIRGEN DEL CARMEN</t>
+        </is>
+      </c>
+      <c r="AG36" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH36" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Huari</t>
         </is>
       </c>
@@ -5132,6 +5492,16 @@
       </c>
       <c r="AF37" t="inlineStr">
         <is>
+          <t>HORACIO GONZALES ESCUDERO</t>
+        </is>
+      </c>
+      <c r="AG37" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH37" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Quinuabamba</t>
         </is>
       </c>
@@ -5254,6 +5624,16 @@
       </c>
       <c r="AF38" t="inlineStr">
         <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH38" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Cochcarcas</t>
         </is>
       </c>
@@ -5376,6 +5756,16 @@
       </c>
       <c r="AF39" t="inlineStr">
         <is>
+          <t>475-3</t>
+        </is>
+      </c>
+      <c r="AG39" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH39" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Cochcarcas</t>
         </is>
       </c>
@@ -5500,6 +5890,16 @@
       </c>
       <c r="AF40" t="inlineStr">
         <is>
+          <t>54481</t>
+        </is>
+      </c>
+      <c r="AG40" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH40" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Cochcarcas</t>
         </is>
       </c>
@@ -5622,6 +6022,16 @@
       </c>
       <c r="AF41" t="inlineStr">
         <is>
+          <t>475-23</t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH41" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Cochcarcas</t>
         </is>
       </c>
@@ -5746,6 +6156,16 @@
       </c>
       <c r="AF42" t="inlineStr">
         <is>
+          <t>MARIO VARGAS LLOSA</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH42" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Cochcarcas</t>
         </is>
       </c>
@@ -5867,6 +6287,16 @@
         </is>
       </c>
       <c r="AF43" t="inlineStr">
+        <is>
+          <t>904</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH43" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Cochcarcas</t>
         </is>
@@ -5978,6 +6408,16 @@
       </c>
       <c r="AF44" t="inlineStr">
         <is>
+          <t>40262 JOSE SEBASTIAN BARRANCA Y LOVERA</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH44" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6088,6 +6528,16 @@
       </c>
       <c r="AF45" t="inlineStr">
         <is>
+          <t>40265</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH45" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6198,6 +6648,16 @@
       </c>
       <c r="AF46" t="inlineStr">
         <is>
+          <t>40308</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH46" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6308,6 +6768,16 @@
       </c>
       <c r="AF47" t="inlineStr">
         <is>
+          <t>41064</t>
+        </is>
+      </c>
+      <c r="AG47" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH47" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6418,6 +6888,16 @@
       </c>
       <c r="AF48" t="inlineStr">
         <is>
+          <t>41507</t>
+        </is>
+      </c>
+      <c r="AG48" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH48" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6528,6 +7008,16 @@
       </c>
       <c r="AF49" t="inlineStr">
         <is>
+          <t>41517</t>
+        </is>
+      </c>
+      <c r="AG49" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH49" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6638,6 +7128,16 @@
       </c>
       <c r="AF50" t="inlineStr">
         <is>
+          <t>EL MOLINO</t>
+        </is>
+      </c>
+      <c r="AG50" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH50" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6748,6 +7248,16 @@
       </c>
       <c r="AF51" t="inlineStr">
         <is>
+          <t>FRANCISCO BOLOGNESI</t>
+        </is>
+      </c>
+      <c r="AG51" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH51" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6858,6 +7368,16 @@
       </c>
       <c r="AF52" t="inlineStr">
         <is>
+          <t>NICOLAS DE PIEROLA/NICOLAS DE PIEROLA</t>
+        </is>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH52" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -6968,6 +7488,16 @@
       </c>
       <c r="AF53" t="inlineStr">
         <is>
+          <t>NIÑOS DE BELEN</t>
+        </is>
+      </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH53" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Acari</t>
         </is>
       </c>
@@ -7099,6 +7629,16 @@
         </is>
       </c>
       <c r="AF54" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH54" t="inlineStr">
         <is>
           <t>Anexo 2 - MP Cangallo</t>
         </is>
@@ -7206,6 +7746,16 @@
       </c>
       <c r="AF55" t="inlineStr">
         <is>
+          <t>24073</t>
+        </is>
+      </c>
+      <c r="AG55" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH55" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Carmen Salcedo</t>
         </is>
       </c>
@@ -7311,6 +7861,16 @@
         </is>
       </c>
       <c r="AF56" t="inlineStr">
+        <is>
+          <t>GLORIOSO AMAUTA</t>
+        </is>
+      </c>
+      <c r="AG56" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH56" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Carmen Salcedo</t>
         </is>
@@ -7410,6 +7970,16 @@
       </c>
       <c r="AF57" t="inlineStr">
         <is>
+          <t>357</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH57" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -7508,6 +8078,16 @@
       </c>
       <c r="AF58" t="inlineStr">
         <is>
+          <t>38397</t>
+        </is>
+      </c>
+      <c r="AG58" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH58" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -7606,6 +8186,16 @@
       </c>
       <c r="AF59" t="inlineStr">
         <is>
+          <t>38374</t>
+        </is>
+      </c>
+      <c r="AG59" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH59" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -7704,6 +8294,16 @@
       </c>
       <c r="AF60" t="inlineStr">
         <is>
+          <t>38375</t>
+        </is>
+      </c>
+      <c r="AG60" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH60" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -7802,6 +8402,16 @@
       </c>
       <c r="AF61" t="inlineStr">
         <is>
+          <t>38376</t>
+        </is>
+      </c>
+      <c r="AG61" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH61" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -7900,6 +8510,16 @@
       </c>
       <c r="AF62" t="inlineStr">
         <is>
+          <t>38413</t>
+        </is>
+      </c>
+      <c r="AG62" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH62" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -7998,6 +8618,16 @@
       </c>
       <c r="AF63" t="inlineStr">
         <is>
+          <t>38720</t>
+        </is>
+      </c>
+      <c r="AG63" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH63" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -8096,6 +8726,16 @@
       </c>
       <c r="AF64" t="inlineStr">
         <is>
+          <t>38764</t>
+        </is>
+      </c>
+      <c r="AG64" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH64" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -8194,6 +8834,16 @@
       </c>
       <c r="AF65" t="inlineStr">
         <is>
+          <t>RAMIRO PRIALE PRIALE</t>
+        </is>
+      </c>
+      <c r="AG65" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH65" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -8292,6 +8942,16 @@
       </c>
       <c r="AF66" t="inlineStr">
         <is>
+          <t>425-1</t>
+        </is>
+      </c>
+      <c r="AG66" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH66" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -8390,6 +9050,16 @@
       </c>
       <c r="AF67" t="inlineStr">
         <is>
+          <t>425-87</t>
+        </is>
+      </c>
+      <c r="AG67" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH67" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -8488,6 +9158,16 @@
       </c>
       <c r="AF68" t="inlineStr">
         <is>
+          <t>425-88</t>
+        </is>
+      </c>
+      <c r="AG68" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH68" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -8586,6 +9266,16 @@
       </c>
       <c r="AF69" t="inlineStr">
         <is>
+          <t>425-89</t>
+        </is>
+      </c>
+      <c r="AG69" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH69" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Chilcas</t>
         </is>
       </c>
@@ -8694,6 +9384,16 @@
       </c>
       <c r="AF70" t="inlineStr">
         <is>
+          <t>FERMIN AVILA</t>
+        </is>
+      </c>
+      <c r="AG70" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH70" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Mi Peru</t>
         </is>
       </c>
@@ -8816,6 +9516,16 @@
       </c>
       <c r="AF71" t="inlineStr">
         <is>
+          <t>MANUEL SEOANE CORRALES/MANUEL SEOANE CORRALES/MANUEL SEOANE CORRALES/MANUEL SEOANE CORRALES</t>
+        </is>
+      </c>
+      <c r="AG71" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH71" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Mi Peru</t>
         </is>
       </c>
@@ -8931,6 +9641,16 @@
         </is>
       </c>
       <c r="AF72" t="inlineStr">
+        <is>
+          <t>FE Y ALEGRIA 33/FE Y ALEGRIA 33/FE Y ALEGRIA 33</t>
+        </is>
+      </c>
+      <c r="AG72" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH72" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Mi Peru</t>
         </is>
@@ -9044,6 +9764,16 @@
       </c>
       <c r="AF73" t="inlineStr">
         <is>
+          <t>5130-4 CHAVINILLO/5130-4</t>
+        </is>
+      </c>
+      <c r="AG73" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH73" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Mi Peru</t>
         </is>
       </c>
@@ -9162,6 +9892,16 @@
       </c>
       <c r="AF74" t="inlineStr">
         <is>
+          <t>LLIHUARI/32728</t>
+        </is>
+      </c>
+      <c r="AG74" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH74" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Maria del Valle</t>
         </is>
       </c>
@@ -9274,6 +10014,16 @@
       </c>
       <c r="AF75" t="inlineStr">
         <is>
+          <t>80201 JULIO RAMON RIBEYRO/80201 JULIO RAMON RIBEYRO/80201 JULIO RAMON RIBEYRO</t>
+        </is>
+      </c>
+      <c r="AG75" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH75" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Marcabal</t>
         </is>
       </c>
@@ -9411,6 +10161,16 @@
         </is>
       </c>
       <c r="AF76" t="inlineStr">
+        <is>
+          <t>80893 NUESTRA SEÑORA DE LA CANDELARIA/80893 NUESTRA SEÑORA DE LA CANDELARIA</t>
+        </is>
+      </c>
+      <c r="AG76" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH76" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Marcabal</t>
         </is>
@@ -9520,6 +10280,16 @@
       </c>
       <c r="AF77" t="inlineStr">
         <is>
+          <t>81625/81625/81625</t>
+        </is>
+      </c>
+      <c r="AG77" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH77" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Marcabal</t>
         </is>
       </c>
@@ -9644,6 +10414,16 @@
       </c>
       <c r="AF78" t="inlineStr">
         <is>
+          <t>1613 MI DULCE HOGAR</t>
+        </is>
+      </c>
+      <c r="AG78" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH78" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Moche</t>
         </is>
       </c>
@@ -9776,6 +10556,16 @@
       </c>
       <c r="AF79" t="inlineStr">
         <is>
+          <t>80082 SAN FRANCISCO DE ASIS</t>
+        </is>
+      </c>
+      <c r="AG79" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH79" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Moche</t>
         </is>
       </c>
@@ -9903,6 +10693,16 @@
         </is>
       </c>
       <c r="AF80" t="inlineStr">
+        <is>
+          <t>10124 NUESTRA SEÑORA DE LOURDES/10124 NUESTRA SEÑORA DE LOURDES</t>
+        </is>
+      </c>
+      <c r="AG80" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH80" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Illimo</t>
         </is>
@@ -10022,6 +10822,16 @@
       </c>
       <c r="AF81" t="inlineStr">
         <is>
+          <t>546 SAN ANTONIO</t>
+        </is>
+      </c>
+      <c r="AG81" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH81" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Huaral</t>
         </is>
       </c>
@@ -10146,6 +10956,16 @@
       </c>
       <c r="AF82" t="inlineStr">
         <is>
+          <t>21559 ANTONIO GRAÑA ELIZALDE/21559 ANTONIO GRAÑA ELIZALDE/21559 ANTONIO GRAÑA ELIZALDE</t>
+        </is>
+      </c>
+      <c r="AG82" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH82" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Huaral</t>
         </is>
       </c>
@@ -10270,6 +11090,16 @@
       </c>
       <c r="AF83" t="inlineStr">
         <is>
+          <t>20407/20407</t>
+        </is>
+      </c>
+      <c r="AG83" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH83" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Huaral</t>
         </is>
       </c>
@@ -10393,6 +11223,16 @@
         </is>
       </c>
       <c r="AF84" t="inlineStr">
+        <is>
+          <t>02 JUAN YSHIZAWA YSHIZAWA/02 JUAN YSHIZAWA YSHIZAWA</t>
+        </is>
+      </c>
+      <c r="AG84" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH84" t="inlineStr">
         <is>
           <t>Anexo 2 - MP Huaral</t>
         </is>
@@ -10502,6 +11342,16 @@
       </c>
       <c r="AF85" t="inlineStr">
         <is>
+          <t>LIBERTADOR SIMON BOLIVAR</t>
+        </is>
+      </c>
+      <c r="AG85" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH85" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Pativilca</t>
         </is>
       </c>
@@ -10632,6 +11482,16 @@
       </c>
       <c r="AF86" t="inlineStr">
         <is>
+          <t>506</t>
+        </is>
+      </c>
+      <c r="AG86" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH86" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Jenaro Herrera</t>
         </is>
       </c>
@@ -10762,6 +11622,16 @@
       </c>
       <c r="AF87" t="inlineStr">
         <is>
+          <t>559</t>
+        </is>
+      </c>
+      <c r="AG87" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH87" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Jenaro Herrera</t>
         </is>
       </c>
@@ -10892,6 +11762,16 @@
       </c>
       <c r="AF88" t="inlineStr">
         <is>
+          <t>60625 GUSTAVO BARTRA VALDIVIEZO/60625 GUSTAVO BARTRA VALDIVIEZO/60625 GUSTAVO BARTRA VALDIVIEZO</t>
+        </is>
+      </c>
+      <c r="AG88" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH88" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Jenaro Herrera</t>
         </is>
       </c>
@@ -11021,6 +11901,16 @@
         </is>
       </c>
       <c r="AF89" t="inlineStr">
+        <is>
+          <t>601005/601005/601005</t>
+        </is>
+      </c>
+      <c r="AG89" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH89" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Jenaro Herrera</t>
         </is>
@@ -11132,6 +12022,16 @@
       </c>
       <c r="AF90" t="inlineStr">
         <is>
+          <t>64249</t>
+        </is>
+      </c>
+      <c r="AG90" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH90" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Pampa Hermosa</t>
         </is>
       </c>
@@ -11264,6 +12164,16 @@
       </c>
       <c r="AF91" t="inlineStr">
         <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="AG91" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH91" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -11396,6 +12306,16 @@
       </c>
       <c r="AF92" t="inlineStr">
         <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="AG92" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH92" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -11528,6 +12448,16 @@
       </c>
       <c r="AF93" t="inlineStr">
         <is>
+          <t>HUATAPI</t>
+        </is>
+      </c>
+      <c r="AG93" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH93" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -11660,6 +12590,16 @@
       </c>
       <c r="AF94" t="inlineStr">
         <is>
+          <t>PUCATE</t>
+        </is>
+      </c>
+      <c r="AG94" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH94" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -11792,6 +12732,16 @@
       </c>
       <c r="AF95" t="inlineStr">
         <is>
+          <t>ESPERANZA</t>
+        </is>
+      </c>
+      <c r="AG95" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH95" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -11924,6 +12874,16 @@
       </c>
       <c r="AF96" t="inlineStr">
         <is>
+          <t>62023</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH96" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -12056,6 +13016,16 @@
       </c>
       <c r="AF97" t="inlineStr">
         <is>
+          <t>ESPERANZA/ESPERANZA</t>
+        </is>
+      </c>
+      <c r="AG97" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH97" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -12188,6 +13158,16 @@
       </c>
       <c r="AF98" t="inlineStr">
         <is>
+          <t>62070</t>
+        </is>
+      </c>
+      <c r="AG98" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH98" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -12320,6 +13300,16 @@
       </c>
       <c r="AF99" t="inlineStr">
         <is>
+          <t>62071</t>
+        </is>
+      </c>
+      <c r="AG99" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH99" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -12452,6 +13442,16 @@
       </c>
       <c r="AF100" t="inlineStr">
         <is>
+          <t>PUCATE</t>
+        </is>
+      </c>
+      <c r="AG100" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH100" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -12584,6 +13584,16 @@
       </c>
       <c r="AF101" t="inlineStr">
         <is>
+          <t>SANTA GEMA/SANTA GEMA</t>
+        </is>
+      </c>
+      <c r="AG101" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH101" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -12716,6 +13726,16 @@
       </c>
       <c r="AF102" t="inlineStr">
         <is>
+          <t>62077</t>
+        </is>
+      </c>
+      <c r="AG102" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH102" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -12848,6 +13868,16 @@
       </c>
       <c r="AF103" t="inlineStr">
         <is>
+          <t>62135/62135/62135</t>
+        </is>
+      </c>
+      <c r="AG103" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH103" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -12980,6 +14010,16 @@
       </c>
       <c r="AF104" t="inlineStr">
         <is>
+          <t>MIGUEL GRAU SEMINARIO</t>
+        </is>
+      </c>
+      <c r="AG104" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH104" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -13112,6 +14152,16 @@
       </c>
       <c r="AF105" t="inlineStr">
         <is>
+          <t>ANGAMOS/ANGAMOS</t>
+        </is>
+      </c>
+      <c r="AG105" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH105" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -13244,6 +14294,16 @@
       </c>
       <c r="AF106" t="inlineStr">
         <is>
+          <t>62254/62254</t>
+        </is>
+      </c>
+      <c r="AG106" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH106" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -13376,6 +14436,16 @@
       </c>
       <c r="AF107" t="inlineStr">
         <is>
+          <t>JOSE OBLITAS HIDALGO</t>
+        </is>
+      </c>
+      <c r="AG107" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH107" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -13508,6 +14578,16 @@
       </c>
       <c r="AF108" t="inlineStr">
         <is>
+          <t>62396</t>
+        </is>
+      </c>
+      <c r="AG108" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH108" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -13640,6 +14720,16 @@
       </c>
       <c r="AF109" t="inlineStr">
         <is>
+          <t>62413/62413</t>
+        </is>
+      </c>
+      <c r="AG109" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH109" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -13772,6 +14862,16 @@
       </c>
       <c r="AF110" t="inlineStr">
         <is>
+          <t>62443/62443/62443</t>
+        </is>
+      </c>
+      <c r="AG110" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH110" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -13904,6 +15004,16 @@
       </c>
       <c r="AF111" t="inlineStr">
         <is>
+          <t>62476/62476</t>
+        </is>
+      </c>
+      <c r="AG111" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH111" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -14036,6 +15146,16 @@
       </c>
       <c r="AF112" t="inlineStr">
         <is>
+          <t>62482/62482</t>
+        </is>
+      </c>
+      <c r="AG112" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH112" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -14168,6 +15288,16 @@
       </c>
       <c r="AF113" t="inlineStr">
         <is>
+          <t>SANTA CRUZ</t>
+        </is>
+      </c>
+      <c r="AG113" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH113" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -14300,6 +15430,16 @@
       </c>
       <c r="AF114" t="inlineStr">
         <is>
+          <t>SANTA GEMA</t>
+        </is>
+      </c>
+      <c r="AG114" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH114" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -14432,6 +15572,16 @@
       </c>
       <c r="AF115" t="inlineStr">
         <is>
+          <t>145</t>
+        </is>
+      </c>
+      <c r="AG115" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH115" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Santa Cruz</t>
         </is>
       </c>
@@ -14548,6 +15698,16 @@
       </c>
       <c r="AF116" t="inlineStr">
         <is>
+          <t>345 BOCA MANU</t>
+        </is>
+      </c>
+      <c r="AG116" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH116" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -14668,6 +15828,16 @@
       </c>
       <c r="AF117" t="inlineStr">
         <is>
+          <t>327</t>
+        </is>
+      </c>
+      <c r="AG117" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH117" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -14788,6 +15958,16 @@
       </c>
       <c r="AF118" t="inlineStr">
         <is>
+          <t>DIAMANTE</t>
+        </is>
+      </c>
+      <c r="AG118" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH118" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -14908,6 +16088,16 @@
       </c>
       <c r="AF119" t="inlineStr">
         <is>
+          <t>52245</t>
+        </is>
+      </c>
+      <c r="AG119" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH119" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15028,6 +16218,16 @@
       </c>
       <c r="AF120" t="inlineStr">
         <is>
+          <t>360</t>
+        </is>
+      </c>
+      <c r="AG120" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH120" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15148,6 +16348,16 @@
       </c>
       <c r="AF121" t="inlineStr">
         <is>
+          <t>364</t>
+        </is>
+      </c>
+      <c r="AG121" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH121" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15260,6 +16470,16 @@
       </c>
       <c r="AF122" t="inlineStr">
         <is>
+          <t>406</t>
+        </is>
+      </c>
+      <c r="AG122" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH122" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15380,6 +16600,16 @@
       </c>
       <c r="AF123" t="inlineStr">
         <is>
+          <t>50843</t>
+        </is>
+      </c>
+      <c r="AG123" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH123" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15500,6 +16730,16 @@
       </c>
       <c r="AF124" t="inlineStr">
         <is>
+          <t>52200</t>
+        </is>
+      </c>
+      <c r="AG124" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH124" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15612,6 +16852,16 @@
       </c>
       <c r="AF125" t="inlineStr">
         <is>
+          <t>52133</t>
+        </is>
+      </c>
+      <c r="AG125" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH125" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15732,6 +16982,16 @@
       </c>
       <c r="AF126" t="inlineStr">
         <is>
+          <t>332 DOCE DE ENERO</t>
+        </is>
+      </c>
+      <c r="AG126" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH126" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15844,6 +17104,16 @@
       </c>
       <c r="AF127" t="inlineStr">
         <is>
+          <t>446</t>
+        </is>
+      </c>
+      <c r="AG127" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH127" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -15956,6 +17226,16 @@
       </c>
       <c r="AF128" t="inlineStr">
         <is>
+          <t>270</t>
+        </is>
+      </c>
+      <c r="AG128" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH128" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -16068,6 +17348,16 @@
       </c>
       <c r="AF129" t="inlineStr">
         <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="AG129" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH129" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -16180,6 +17470,16 @@
       </c>
       <c r="AF130" t="inlineStr">
         <is>
+          <t>308</t>
+        </is>
+      </c>
+      <c r="AG130" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH130" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -16300,6 +17600,16 @@
       </c>
       <c r="AF131" t="inlineStr">
         <is>
+          <t>53004 MIGUEL GRAU</t>
+        </is>
+      </c>
+      <c r="AG131" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH131" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -16420,6 +17730,16 @@
       </c>
       <c r="AF132" t="inlineStr">
         <is>
+          <t>EL ARCA DE PACAHUARA/52216 EL ARCA DE PACAHUARA</t>
+        </is>
+      </c>
+      <c r="AG132" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH132" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -16540,6 +17860,16 @@
       </c>
       <c r="AF133" t="inlineStr">
         <is>
+          <t>392</t>
+        </is>
+      </c>
+      <c r="AG133" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH133" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -16656,6 +17986,16 @@
       </c>
       <c r="AF134" t="inlineStr">
         <is>
+          <t>335</t>
+        </is>
+      </c>
+      <c r="AG134" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH134" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -16768,6 +18108,16 @@
       </c>
       <c r="AF135" t="inlineStr">
         <is>
+          <t>412</t>
+        </is>
+      </c>
+      <c r="AG135" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH135" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -16884,6 +18234,16 @@
       </c>
       <c r="AF136" t="inlineStr">
         <is>
+          <t>275</t>
+        </is>
+      </c>
+      <c r="AG136" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH136" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -17000,6 +18360,16 @@
       </c>
       <c r="AF137" t="inlineStr">
         <is>
+          <t>52077/52077</t>
+        </is>
+      </c>
+      <c r="AG137" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH137" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -17116,6 +18486,16 @@
       </c>
       <c r="AF138" t="inlineStr">
         <is>
+          <t>52129</t>
+        </is>
+      </c>
+      <c r="AG138" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH138" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -17236,6 +18616,16 @@
       </c>
       <c r="AF139" t="inlineStr">
         <is>
+          <t>RICARDO PALMA SORIANO/52187 RICARDO PALMA SORIANO</t>
+        </is>
+      </c>
+      <c r="AG139" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH139" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -17352,6 +18742,16 @@
       </c>
       <c r="AF140" t="inlineStr">
         <is>
+          <t>366</t>
+        </is>
+      </c>
+      <c r="AG140" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH140" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -17472,6 +18872,16 @@
       </c>
       <c r="AF141" t="inlineStr">
         <is>
+          <t>368 NIÑOS DE LA SELVA</t>
+        </is>
+      </c>
+      <c r="AG141" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH141" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -17592,6 +19002,16 @@
       </c>
       <c r="AF142" t="inlineStr">
         <is>
+          <t>388</t>
+        </is>
+      </c>
+      <c r="AG142" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH142" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -17708,6 +19128,16 @@
       </c>
       <c r="AF143" t="inlineStr">
         <is>
+          <t>NUEVA AREQUIPA</t>
+        </is>
+      </c>
+      <c r="AG143" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH143" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -17828,6 +19258,16 @@
       </c>
       <c r="AF144" t="inlineStr">
         <is>
+          <t>52055</t>
+        </is>
+      </c>
+      <c r="AG144" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH144" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -17948,6 +19388,16 @@
       </c>
       <c r="AF145" t="inlineStr">
         <is>
+          <t>IÑAPARI</t>
+        </is>
+      </c>
+      <c r="AG145" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH145" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -18068,6 +19518,16 @@
       </c>
       <c r="AF146" t="inlineStr">
         <is>
+          <t>394</t>
+        </is>
+      </c>
+      <c r="AG146" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH146" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -18188,6 +19648,16 @@
       </c>
       <c r="AF147" t="inlineStr">
         <is>
+          <t>52062 JAVIER HERAUD/52062 JAVIER HERAUD</t>
+        </is>
+      </c>
+      <c r="AG147" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH147" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -18308,6 +19778,16 @@
       </c>
       <c r="AF148" t="inlineStr">
         <is>
+          <t>52033/52033</t>
+        </is>
+      </c>
+      <c r="AG148" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH148" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -18420,6 +19900,16 @@
       </c>
       <c r="AF149" t="inlineStr">
         <is>
+          <t>52105</t>
+        </is>
+      </c>
+      <c r="AG149" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH149" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -18540,6 +20030,16 @@
       </c>
       <c r="AF150" t="inlineStr">
         <is>
+          <t>328</t>
+        </is>
+      </c>
+      <c r="AG150" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH150" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -18660,6 +20160,16 @@
       </c>
       <c r="AF151" t="inlineStr">
         <is>
+          <t>JAVIER HERAUD</t>
+        </is>
+      </c>
+      <c r="AG151" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH151" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -18780,6 +20290,16 @@
       </c>
       <c r="AF152" t="inlineStr">
         <is>
+          <t>52262 CARLOS MARQUEZ BRAGA</t>
+        </is>
+      </c>
+      <c r="AG152" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH152" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -18900,6 +20420,16 @@
       </c>
       <c r="AF153" t="inlineStr">
         <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="AG153" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH153" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19012,6 +20542,16 @@
       </c>
       <c r="AF154" t="inlineStr">
         <is>
+          <t>HEROES DE ILLAMPU/HEROES DE ILLAMPU/HEROES DE ILLAMPU</t>
+        </is>
+      </c>
+      <c r="AG154" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH154" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19132,6 +20672,16 @@
       </c>
       <c r="AF155" t="inlineStr">
         <is>
+          <t>52095/52095</t>
+        </is>
+      </c>
+      <c r="AG155" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH155" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19252,6 +20802,16 @@
       </c>
       <c r="AF156" t="inlineStr">
         <is>
+          <t>52136</t>
+        </is>
+      </c>
+      <c r="AG156" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH156" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19372,6 +20932,16 @@
       </c>
       <c r="AF157" t="inlineStr">
         <is>
+          <t>52242</t>
+        </is>
+      </c>
+      <c r="AG157" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH157" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19492,6 +21062,16 @@
       </c>
       <c r="AF158" t="inlineStr">
         <is>
+          <t>52137</t>
+        </is>
+      </c>
+      <c r="AG158" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH158" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19612,6 +21192,16 @@
       </c>
       <c r="AF159" t="inlineStr">
         <is>
+          <t>396</t>
+        </is>
+      </c>
+      <c r="AG159" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH159" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19724,6 +21314,16 @@
       </c>
       <c r="AF160" t="inlineStr">
         <is>
+          <t>413</t>
+        </is>
+      </c>
+      <c r="AG160" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH160" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19840,6 +21440,16 @@
       </c>
       <c r="AF161" t="inlineStr">
         <is>
+          <t>52081</t>
+        </is>
+      </c>
+      <c r="AG161" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH161" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -19960,6 +21570,16 @@
       </c>
       <c r="AF162" t="inlineStr">
         <is>
+          <t>52075</t>
+        </is>
+      </c>
+      <c r="AG162" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH162" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -20080,6 +21700,16 @@
       </c>
       <c r="AF163" t="inlineStr">
         <is>
+          <t>52154</t>
+        </is>
+      </c>
+      <c r="AG163" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH163" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -20200,6 +21830,16 @@
       </c>
       <c r="AF164" t="inlineStr">
         <is>
+          <t>PEDRO PAULET/PEDRO PAULET</t>
+        </is>
+      </c>
+      <c r="AG164" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH164" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -20312,6 +21952,16 @@
       </c>
       <c r="AF165" t="inlineStr">
         <is>
+          <t>325</t>
+        </is>
+      </c>
+      <c r="AG165" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH165" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -20432,6 +22082,16 @@
       </c>
       <c r="AF166" t="inlineStr">
         <is>
+          <t>DANIEL ALCIDES CARRION/DANIEL ALCIDES CARRION</t>
+        </is>
+      </c>
+      <c r="AG166" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH166" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -20552,6 +22212,16 @@
       </c>
       <c r="AF167" t="inlineStr">
         <is>
+          <t>393</t>
+        </is>
+      </c>
+      <c r="AG167" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH167" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -20664,6 +22334,16 @@
       </c>
       <c r="AF168" t="inlineStr">
         <is>
+          <t>279 NIÑO DE PRAGA</t>
+        </is>
+      </c>
+      <c r="AG168" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH168" t="inlineStr">
+        <is>
           <t>Anexo 2 - GORE Madre de Dios</t>
         </is>
       </c>
@@ -20784,6 +22464,16 @@
       </c>
       <c r="AF169" t="inlineStr">
         <is>
+          <t>52061/52061</t>
+        </is>
+      </c>
+      <c r="AG169" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH169" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Tahuamanu</t>
         </is>
       </c>
@@ -20896,6 +22586,16 @@
       </c>
       <c r="AF170" t="inlineStr">
         <is>
+          <t>389</t>
+        </is>
+      </c>
+      <c r="AG170" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH170" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Tahuamanu</t>
         </is>
       </c>
@@ -21008,6 +22708,16 @@
       </c>
       <c r="AF171" t="inlineStr">
         <is>
+          <t>432</t>
+        </is>
+      </c>
+      <c r="AG171" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH171" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Tahuamanu</t>
         </is>
       </c>
@@ -21128,6 +22838,16 @@
       </c>
       <c r="AF172" t="inlineStr">
         <is>
+          <t>266</t>
+        </is>
+      </c>
+      <c r="AG172" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH172" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -21248,6 +22968,16 @@
       </c>
       <c r="AF173" t="inlineStr">
         <is>
+          <t>296 LAS PALMERAS</t>
+        </is>
+      </c>
+      <c r="AG173" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH173" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -21368,6 +23098,16 @@
       </c>
       <c r="AF174" t="inlineStr">
         <is>
+          <t>297</t>
+        </is>
+      </c>
+      <c r="AG174" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH174" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -21488,6 +23228,16 @@
       </c>
       <c r="AF175" t="inlineStr">
         <is>
+          <t>307</t>
+        </is>
+      </c>
+      <c r="AG175" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH175" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -21608,6 +23358,16 @@
       </c>
       <c r="AF176" t="inlineStr">
         <is>
+          <t>312</t>
+        </is>
+      </c>
+      <c r="AG176" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH176" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -21728,6 +23488,16 @@
       </c>
       <c r="AF177" t="inlineStr">
         <is>
+          <t>313</t>
+        </is>
+      </c>
+      <c r="AG177" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH177" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -21840,6 +23610,16 @@
       </c>
       <c r="AF178" t="inlineStr">
         <is>
+          <t>318 MI PEQUEÑO MUNDO</t>
+        </is>
+      </c>
+      <c r="AG178" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH178" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -21960,6 +23740,16 @@
       </c>
       <c r="AF179" t="inlineStr">
         <is>
+          <t>LA PASTORA/LA PASTORA/LA PASTORA</t>
+        </is>
+      </c>
+      <c r="AG179" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH179" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -22080,6 +23870,16 @@
       </c>
       <c r="AF180" t="inlineStr">
         <is>
+          <t>SAN BERNARDO/52035</t>
+        </is>
+      </c>
+      <c r="AG180" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH180" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -22200,6 +24000,16 @@
       </c>
       <c r="AF181" t="inlineStr">
         <is>
+          <t>52084</t>
+        </is>
+      </c>
+      <c r="AG181" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH181" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -22320,6 +24130,16 @@
       </c>
       <c r="AF182" t="inlineStr">
         <is>
+          <t>52166 NUESTRA SEÑORA DE FATIMA/52166 NUESTRA SEÑORA DE FATIMA</t>
+        </is>
+      </c>
+      <c r="AG182" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH182" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -22440,6 +24260,16 @@
       </c>
       <c r="AF183" t="inlineStr">
         <is>
+          <t>433 ROBERTO GUILLERMO VELA VALLES/52183/52183</t>
+        </is>
+      </c>
+      <c r="AG183" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH183" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -22552,6 +24382,16 @@
       </c>
       <c r="AF184" t="inlineStr">
         <is>
+          <t>SANTA RITA DE CASIA</t>
+        </is>
+      </c>
+      <c r="AG184" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH184" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -22672,6 +24512,16 @@
       </c>
       <c r="AF185" t="inlineStr">
         <is>
+          <t>52225</t>
+        </is>
+      </c>
+      <c r="AG185" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH185" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -22792,6 +24642,16 @@
       </c>
       <c r="AF186" t="inlineStr">
         <is>
+          <t>52028</t>
+        </is>
+      </c>
+      <c r="AG186" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH186" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -22912,6 +24772,16 @@
       </c>
       <c r="AF187" t="inlineStr">
         <is>
+          <t>395</t>
+        </is>
+      </c>
+      <c r="AG187" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH187" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -23032,6 +24902,16 @@
       </c>
       <c r="AF188" t="inlineStr">
         <is>
+          <t>398</t>
+        </is>
+      </c>
+      <c r="AG188" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH188" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -23144,6 +25024,16 @@
       </c>
       <c r="AF189" t="inlineStr">
         <is>
+          <t>400 LUCECITAS DEL SABER</t>
+        </is>
+      </c>
+      <c r="AG189" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH189" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -23264,6 +25154,16 @@
       </c>
       <c r="AF190" t="inlineStr">
         <is>
+          <t>292</t>
+        </is>
+      </c>
+      <c r="AG190" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH190" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -23384,6 +25284,16 @@
       </c>
       <c r="AF191" t="inlineStr">
         <is>
+          <t>52028</t>
+        </is>
+      </c>
+      <c r="AG191" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH191" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tambopata</t>
         </is>
       </c>
@@ -23516,6 +25426,16 @@
       </c>
       <c r="AF192" t="inlineStr">
         <is>
+          <t>14857 SAN MIGUEL ARCANGEL</t>
+        </is>
+      </c>
+      <c r="AG192" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH192" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Sullana</t>
         </is>
       </c>
@@ -23631,6 +25551,16 @@
         </is>
       </c>
       <c r="AF193" t="inlineStr">
+        <is>
+          <t>POSIC/POSIC</t>
+        </is>
+      </c>
+      <c r="AG193" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH193" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Posic</t>
         </is>
@@ -23740,6 +25670,16 @@
       </c>
       <c r="AF194" t="inlineStr">
         <is>
+          <t>POSIC/POSIC</t>
+        </is>
+      </c>
+      <c r="AG194" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH194" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Posic</t>
         </is>
       </c>
@@ -23844,6 +25784,16 @@
       </c>
       <c r="AF195" t="inlineStr">
         <is>
+          <t>291</t>
+        </is>
+      </c>
+      <c r="AG195" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH195" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Yorongos</t>
         </is>
       </c>
@@ -23948,6 +25898,16 @@
       </c>
       <c r="AF196" t="inlineStr">
         <is>
+          <t>00553 JUANA MORI VELA</t>
+        </is>
+      </c>
+      <c r="AG196" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH196" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Yorongos</t>
         </is>
       </c>
@@ -24052,6 +26012,16 @@
       </c>
       <c r="AF197" t="inlineStr">
         <is>
+          <t>00897</t>
+        </is>
+      </c>
+      <c r="AG197" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH197" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Yorongos</t>
         </is>
       </c>
@@ -24156,6 +26126,16 @@
       </c>
       <c r="AF198" t="inlineStr">
         <is>
+          <t>00861/00861</t>
+        </is>
+      </c>
+      <c r="AG198" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH198" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Yorongos</t>
         </is>
       </c>
@@ -24260,6 +26240,16 @@
       </c>
       <c r="AF199" t="inlineStr">
         <is>
+          <t>00900</t>
+        </is>
+      </c>
+      <c r="AG199" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH199" t="inlineStr">
+        <is>
           <t>Anexo 2 - MD Yorongos</t>
         </is>
       </c>
@@ -24363,6 +26353,16 @@
         </is>
       </c>
       <c r="AF200" t="inlineStr">
+        <is>
+          <t>WILFREDO EZEQUIEL PONCE CHIRINOS</t>
+        </is>
+      </c>
+      <c r="AG200" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH200" t="inlineStr">
         <is>
           <t>Anexo 2 - MD Yorongos</t>
         </is>
@@ -24472,6 +26472,16 @@
       </c>
       <c r="AF201" t="inlineStr">
         <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="AG201" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH201" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tacna</t>
         </is>
       </c>
@@ -24579,6 +26589,16 @@
         </is>
       </c>
       <c r="AF202" t="inlineStr">
+        <is>
+          <t>354 VIRGEN MARIA</t>
+        </is>
+      </c>
+      <c r="AG202" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH202" t="inlineStr">
         <is>
           <t>Anexo 2 - MP Tacna</t>
         </is>
@@ -24684,6 +26704,16 @@
       </c>
       <c r="AF203" t="inlineStr">
         <is>
+          <t>42053 BARTOLOME JULIO ROSPIGLIOSI</t>
+        </is>
+      </c>
+      <c r="AG203" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH203" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tacna</t>
         </is>
       </c>
@@ -24788,6 +26818,16 @@
       </c>
       <c r="AF204" t="inlineStr">
         <is>
+          <t>42032 JOSE JOAQUIN INCLAN/42032 JOSE JOAQUIN INCLAN</t>
+        </is>
+      </c>
+      <c r="AG204" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH204" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tacna</t>
         </is>
       </c>
@@ -24892,6 +26932,16 @@
       </c>
       <c r="AF205" t="inlineStr">
         <is>
+          <t>443 SANTA TERESITA/443 SANTA TERESITA</t>
+        </is>
+      </c>
+      <c r="AG205" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH205" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tacna</t>
         </is>
       </c>
@@ -24996,6 +27046,16 @@
       </c>
       <c r="AF206" t="inlineStr">
         <is>
+          <t>454</t>
+        </is>
+      </c>
+      <c r="AG206" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="AH206" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tacna</t>
         </is>
       </c>
@@ -25098,6 +27158,16 @@
       </c>
       <c r="AF207" t="inlineStr">
         <is>
+          <t>42010 SANTISIMA NIÑA MARIA/42010 SANTISIMA NIÑA MARIA</t>
+        </is>
+      </c>
+      <c r="AG207" t="inlineStr">
+        <is>
+          <t>Urbana</t>
+        </is>
+      </c>
+      <c r="AH207" t="inlineStr">
+        <is>
           <t>Anexo 2 - MP Tacna</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Canoniza variables, consolidados por grupo y reestructura tipo/fechas
- Diccionario y bases con nombres de variable CANONIZADOS (minuscula/snake_case;
  p.ej. 'Codigo Unico de Inversiones' -> cui). Diccionario muestra variable
  canonica + nombre_original.
- Base consolidada por cada uno de los 11 grupos (conserva todos los campos).
- Grupo 2 (PI): fuente = campo fuentes_concat; cod_mod completado con los
  modulos del local (padron/vinculaciones, 95.8%).
- tipo_intervencion = nombre del grupo (PI = tipo de inversion, 100%); nuevo
  campo tipo_activo = activo intervenido (PI = tipo_intervencion_detectada).
- Reemplaza 'fecha' por fecha_inicio y fecha_fin (o entrega estimada).
- Guardado parquet preserva tipos numericos (sin fallback a string).

https://claude.ai/code/session_01N9afypBcQVKYhttom8P34Z
</commit_message>
<xml_diff>
--- a/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_anexo2_b.xlsx
+++ b/output/bases_limpias/Grupo_01_MOBILIARIO_Y_EQUIPO/df_anexo2_b.xlsx
@@ -423,137 +423,137 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>N°</t>
+          <t>n</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Código local</t>
+          <t>cod_local</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Región</t>
+          <t>departamento</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Provincia</t>
+          <t>provincia</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Distrito</t>
+          <t>distrito</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Nombre de la I.E.</t>
+          <t>nombre_ie</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>1. Cantidad de mobiliarios - Aulas</t>
+          <t>1_cantidad_de_mobiliarios_aulas</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>1. Año de intervención de mobiliario - Aulas</t>
+          <t>1_ano_de_intervencion_de_mobiliario_aulas</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>2. Cantidad de mobiliario - Aula de Innovación Pedagógica</t>
+          <t>2_cantidad_de_mobiliario_aula_de_innovacion_pedagogica</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>2. Año de intervención de mobiliario - Aula de Innovación Pedagógica</t>
+          <t>2_ano_de_intervencion_de_mobiliario_aula_de_innovacion_pedag</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>2. Cantidad de mobiliarios - otros ambientes</t>
+          <t>2_cantidad_de_mobiliarios_otros_ambientes</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>3. Describir los ambientes intervenidos</t>
+          <t>3_describir_los_ambientes_intervenidos</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>3. Año de intervención de mobiliarios - otros ambientes</t>
+          <t>3_ano_de_intervencion_de_mobiliarios_otros_ambientes</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Monto contractual total de mobiliarios (S/)</t>
+          <t>monto_contractual_total_de_mobiliarios_s</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>1. Cantidad de equipamiento - Aulas</t>
+          <t>1_cantidad_de_equipamiento_aulas</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>1. Año de intervención de equipamiento - Aulas</t>
+          <t>1_ano_de_intervencion_de_equipamiento_aulas</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>2. Cantidad de equipamiento - Aula de Innovación Pedagógica</t>
+          <t>2_cantidad_de_equipamiento_aula_de_innovacion_pedagogica</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>2. Año de intervención de equipamiento - Aula de Innovación Pedagógica</t>
+          <t>2_ano_de_intervencion_de_equipamiento_aula_de_innovacion_ped</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>2. Cantidad de equipamiento - otros ambientes</t>
+          <t>2_cantidad_de_equipamiento_otros_ambientes</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>2. Describir los ambientes intervenidos</t>
+          <t>2_describir_los_ambientes_intervenidos</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>2. Año de intervención de equipamiento - otros ambientes</t>
+          <t>2_ano_de_intervencion_de_equipamiento_otros_ambientes</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Monto contractual total de equipamiento (S/)</t>
+          <t>monto_contractual_total_de_equipamiento_s</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Comentarios</t>
+          <t>comentario</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>REMITENTE</t>
+          <t>remitente</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>departamento</t>
+          <t>departamento_2</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>provincia</t>
+          <t>provincia_2</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>distrito</t>
+          <t>distrito_2</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
-          <t>nombre_ie</t>
+          <t>nombre_ie_2</t>
         </is>
       </c>
       <c r="AG1" t="inlineStr">

</xml_diff>